<commit_message>
Papyrus evidence pack for release 0.1.0+a3d9ded
Image ghcr.io/beaglabs/papyrus/papyrus@sha256:83b1fb85 (built 2026-10-27): signature and SLSA
provenance verified, no critical or high findings on either platform. Adds the AI RMF mapping
and the capabilities overview, with their build scripts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/compliance/papyrus/papyrus-poam.xlsx
+++ b/public/compliance/papyrus/papyrus-poam.xlsx
@@ -5,7 +5,7 @@
     <sheet name="POA&amp;M" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'POA&amp;M'!$A$1:$K$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'POA&amp;M'!$A$1:$K$32</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -135,17 +135,17 @@
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-3</t>
+          <t xml:space="preserve">AC-2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-3 Access Enforcement</t>
+          <t xml:space="preserve">AC-2 Account Management</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Agent sessions, their messages, the AgentFS Library and generated artifacts are owned by the tenant, not by the person who created them. Any signed-in person holding any Papyrus role can list and read every session, Library file and artifact in the deployment.</t>
+          <t xml:space="preserve">A person who holds System Owner through a Papyrus role assignment keeps access while SCIM reports them deprovisioned (intended as break-glass), and there is no administrator action to end a person's active sessions.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
@@ -155,7 +155,7 @@
       </c>
       <c r="F2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="2">
@@ -165,12 +165,12 @@
       </c>
       <c r="H2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Record an owner on each session and Library namespace, enforce owner or explicit-share checks in the session, workspace-file and artifact routes, and add tests for cross-user denial.</t>
+          <t xml:space="preserve">Limit the SCIM bypass to accounts named in papyrus.yaml and audit each use; add a System Owner action to revoke a person's sessions.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Before first federal ATO package</t>
         </is>
       </c>
       <c r="J2" t="inlineStr" s="2">
@@ -192,17 +192,17 @@
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-4</t>
+          <t xml:space="preserve">AC-3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-4 Information Flow Enforcement</t>
+          <t xml:space="preserve">AC-3 Access Enforcement</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Outbound HTTP from workflow http-get/http-post steps and imported API tools is allowed to any public HTTPS host by default; the organization can block hosts with a denylist but there is no allow-list-only mode.</t>
+          <t xml:space="preserve">Agent sessions, their messages, the AgentFS Library and generated artifacts are owned by the tenant, not by the person who created them. Any signed-in person holding any Papyrus role can list and read every session, Library file and artifact in the deployment.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
@@ -212,7 +212,7 @@
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="2">
@@ -222,7 +222,7 @@
       </c>
       <c r="H3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add an allow-list mode (deny by default) for workflow and imported-API egress, selectable per deployment profile and on by default for the government and disconnected profiles.</t>
+          <t xml:space="preserve">Record an owner on each session and Library namespace, enforce owner or explicit-share checks in the session, workspace-file and artifact routes, and add tests for cross-user denial.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr" s="2">
@@ -249,17 +249,17 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-5</t>
+          <t xml:space="preserve">AC-4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-5 Separation of Duties</t>
+          <t xml:space="preserve">AC-4 Information Flow Enforcement</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Action proposals and governed changes do not check that the approver differs from the person who proposed or requested them, so one person holding the approving roles can approve their own request. Unaddressed workflow approval steps can be answered by the run's initiator.</t>
+          <t xml:space="preserve">Model gateway, identity provider discovery and Sentry connections do not pass the egress gate (they are configured endpoints), and the gate does not pin the resolved address, so a host that changes its DNS answer between check and connect could reach an internal address.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
@@ -269,7 +269,7 @@
       </c>
       <c r="F4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="2">
@@ -279,12 +279,12 @@
       </c>
       <c r="H4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Refuse approval when the approver's object ID equals the proposer or requester for action proposals, governed changes and unaddressed workflow steps, with an explicit single-operator override recorded in the audit log.</t>
+          <t xml:space="preserve">Route every outbound connection through the gate and connect to the address that was checked.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Before first federal ATO package</t>
         </is>
       </c>
       <c r="J4" t="inlineStr" s="2">
@@ -306,17 +306,17 @@
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-6</t>
+          <t xml:space="preserve">AC-5</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-6 Least Privilege</t>
+          <t xml:space="preserve">AC-5 Separation of Duties</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possession of any role, including narrow ones such as Papyrus.Audit.View, grants access to the shared agent workspace: all sessions, chat, Library files and artifacts. Workspace access is not itself a separately assignable privilege.</t>
+          <t xml:space="preserve">Action proposals and governed changes do not check that the approver differs from the person who proposed or requested them, so one person holding the approving roles can approve their own request. Unaddressed workflow approval steps can be answered by the run's initiator.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="2">
@@ -326,7 +326,7 @@
       </c>
       <c r="F5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="2">
@@ -336,7 +336,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Introduce a distinct workspace-use role or per-session ownership (see ac-3) so that narrow roles do not carry workspace access.</t>
+          <t xml:space="preserve">Refuse approval when the approver's object ID equals the proposer or requester for action proposals, governed changes and unaddressed workflow steps, with an explicit single-operator override recorded in the audit log.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="2">
@@ -363,17 +363,17 @@
       </c>
       <c r="B6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-12</t>
+          <t xml:space="preserve">AC-6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AC-12 Session Termination</t>
+          <t xml:space="preserve">AC-6 Least Privilege</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sessions are stateless: there is no server-side session store, idle timeout, or revocation list. A copied cookie remains valid until its one-hour expiry after sign-out, and on deployments using their own app registration the roles carried in the cookie persist until expiry after an Entra role is removed.</t>
+          <t xml:space="preserve">Possession of any role, including narrow ones such as Papyrus.Audit.View, grants access to the shared agent workspace: all sessions, chat, Library files and artifacts. Workspace access is not itself a separately assignable privilege.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="2">
@@ -383,7 +383,7 @@
       </c>
       <c r="F6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="2">
@@ -393,12 +393,12 @@
       </c>
       <c r="H6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add a server-side session table with idle timeout, explicit revocation on sign-out, and an administrator action to end a person's sessions.</t>
+          <t xml:space="preserve">Introduce a distinct workspace-use role or per-session ownership (see ac-3) so that narrow roles do not carry workspace access.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Before first federal pilot</t>
         </is>
       </c>
       <c r="J6" t="inlineStr" s="2">
@@ -420,17 +420,17 @@
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-2</t>
+          <t xml:space="preserve">AC-16</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-2 Event Logging</t>
+          <t xml:space="preserve">AC-16 Security and Privacy Attributes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Successful and failed sign-ins and authorization denials (401/403) are not written to a local audit record. A successful sign-in is only sent as an analytics event to Beag Labs on registered deployments.</t>
+          <t xml:space="preserve">Files Papyrus generates (PDF, DOCX, XLSX, exports) are not marked, and records carry no per-item classification.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="2">
@@ -440,7 +440,7 @@
       </c>
       <c r="F7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G7" t="inlineStr" s="2">
@@ -450,12 +450,12 @@
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Write sign-in success, sign-in failure and authorization-denied events to an append-only local audit table with actor, time, route and outcome.</t>
+          <t xml:space="preserve">Stamp the system-high marking on generated files and exports.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J7" t="inlineStr" s="2">
@@ -477,17 +477,17 @@
       </c>
       <c r="B8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-3</t>
+          <t xml:space="preserve">AU-2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-3 Content of Audit Records</t>
+          <t xml:space="preserve">AU-2 Event Logging</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Audit records do not capture the client network address, and each log uses its own schema, so records cannot be correlated or exported in one format.</t>
+          <t xml:space="preserve">Document downloads, session and workflow deletions, and agent tool calls are recorded in their own stores or not at all, rather than in the unified audit trail.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="2">
@@ -497,7 +497,7 @@
       </c>
       <c r="F8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="2">
@@ -507,17 +507,17 @@
       </c>
       <c r="H8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add source address and request ID to audit writes and define a common audit event schema used by all append-only logs.</t>
+          <t xml:space="preserve">Write these events to the unified audit trail.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Next release</t>
         </is>
       </c>
       <c r="J8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">low</t>
+          <t xml:space="preserve">moderate</t>
         </is>
       </c>
       <c r="K8" t="inlineStr" s="2">
@@ -534,17 +534,17 @@
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-6</t>
+          <t xml:space="preserve">AU-4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AU-6 Audit Record Review, Analysis, and Reporting</t>
+          <t xml:space="preserve">AU-4 Audit Log Storage Capacity</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">There is no consolidated audit view and no export or forwarding of audit records to an external log store or SIEM; records stay in local SQLite databases.</t>
+          <t xml:space="preserve">Papyrus does not watch free space on the data volume or alert when it runs low.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="2">
@@ -554,7 +554,7 @@
       </c>
       <c r="F9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G9" t="inlineStr" s="2">
@@ -564,17 +564,17 @@
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Provide an audit export API and a streaming forwarder (syslog or OTLP) covering all append-only logs.</t>
+          <t xml:space="preserve">Add capacity monitoring and an alert.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Next release</t>
         </is>
       </c>
       <c r="J9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">moderate</t>
+          <t xml:space="preserve">low</t>
         </is>
       </c>
       <c r="K9" t="inlineStr" s="2">
@@ -601,7 +601,7 @@
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Triggers and the hash chain detect changes made through the application only; anyone with write access to the database file can rewrite them. Chain verification is not exposed through any API or run on a schedule, and logs other than integration and action events are not hash-chained.</t>
+          <t xml:space="preserve">Triggers detect changes made through the application only; anyone with write access to the database file can rewrite local records, and the unified trail is not hash-chained or signed. Off-host export mitigates this only when configured.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="2">
@@ -611,7 +611,7 @@
       </c>
       <c r="F10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G10" t="inlineStr" s="2">
@@ -621,7 +621,7 @@
       </c>
       <c r="H10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Expose chain verification to Audit Viewers, run it periodically, extend chaining to all audit tables, and anchor chain heads in external storage.</t>
+          <t xml:space="preserve">Chain and sign the unified trail with a key held outside the data directory and verify it on a schedule; require OTLP export on classified deployments.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr" s="2">
@@ -668,7 +668,7 @@
       </c>
       <c r="F11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="2">
@@ -725,7 +725,7 @@
       </c>
       <c r="F12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="2">
@@ -782,7 +782,7 @@
       </c>
       <c r="F13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="2">
@@ -819,17 +819,17 @@
       </c>
       <c r="B14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RA-5</t>
+          <t xml:space="preserve">IA-2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RA-5 Vulnerability Monitoring and Scanning</t>
+          <t xml:space="preserve">IA-2 Identification and Authentication (Organizational Users)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No dependency, static-analysis or image vulnerability scanning runs in CI, and there is no Dependabot or equivalent configuration.</t>
+          <t xml:space="preserve">Papyrus does not itself require multi-factor or certificate-based authentication (it trusts the identity provider's policy) and cannot accept client certificates (CAC/PIV or SIPR tokens) directly.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="2">
@@ -839,7 +839,7 @@
       </c>
       <c r="F14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="2">
@@ -849,17 +849,17 @@
       </c>
       <c r="H14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add image and dependency scanning (for example Grype or Trivy against the CycloneDX SBOM) and static analysis to CI, failing builds on critical findings, and enable automated dependency update pull requests.</t>
+          <t xml:space="preserve">Optionally require MFA or smart-card authentication methods in the token (amr/acr), and support mutual TLS with NSS PKI where the enclave requires it.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Next release</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">high</t>
+          <t xml:space="preserve">moderate</t>
         </is>
       </c>
       <c r="K14" t="inlineStr" s="2">
@@ -876,17 +876,17 @@
       </c>
       <c r="B15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SA-9</t>
+          <t xml:space="preserve">RA-5</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SA-9 External System Services</t>
+          <t xml:space="preserve">RA-5 Vulnerability Monitoring and Scanning</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">On registered deployments the server sends each person's Entra object ID, display name and tenant ID to Beag Labs as analytics on sign-in, and there is no setting to turn analytics off separately from registration. Deployments on the government profile register with Beag Labs unless PAPYRUS_BEAGLABS_REGISTRATION=0 is set. Several outbound destinations (embedding download, package registries) are not listed in docs/deployment.md. The control plane and license authority are not in this repository and are not covered by this assessment.</t>
+          <t xml:space="preserve">No dependency or static-analysis scanning runs in CI, and there are no severity-based remediation timeframes.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="2">
@@ -896,7 +896,7 @@
       </c>
       <c r="F15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G15" t="inlineStr" s="2">
@@ -906,7 +906,7 @@
       </c>
       <c r="H15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add a separate analytics opt-out and stop sending display names, default registration off for the government profile, document every outbound destination with its switch, and publish a security description of the control plane and license authority.</t>
+          <t xml:space="preserve">Add dependency and code scanning to CI and publish remediation timeframes.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr" s="2">
@@ -916,7 +916,7 @@
       </c>
       <c r="J15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">moderate</t>
+          <t xml:space="preserve">high</t>
         </is>
       </c>
       <c r="K15" t="inlineStr" s="2">
@@ -943,7 +943,7 @@
       </c>
       <c r="D16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Most security tests, including identity, MCP, Resource Class intake, Key Vault, broker and control-plane tests, do not run in CI, and the compliance drift check runs only in the local pre-commit hook, which can be skipped. compliance/ssp.md states that these checks run in CI.</t>
+          <t xml:space="preserve">Most security tests, including identity, MCP and Key Vault tests, do not run in CI, and the compliance drift check runs only in the local pre-commit hook, which can be skipped. compliance/ssp.md states that these checks run in CI.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="2">
@@ -953,7 +953,7 @@
       </c>
       <c r="F16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G16" t="inlineStr" s="2">
@@ -990,17 +990,17 @@
       </c>
       <c r="B17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-5</t>
+          <t xml:space="preserve">SC-4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-5 Denial-of-Service Protection</t>
+          <t xml:space="preserve">SC-4 Information in Shared System Resources</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Rate limits are in memory and keyed on the socket address; behind the appliance's nginx proxy every client shares one address, and the limiter clears all windows once it tracks 10,000 keys. The cap of 256 pending sign-ins can be exhausted by unauthenticated requests, blocking sign-in for up to 10 minutes.</t>
+          <t xml:space="preserve">Deleting a session does not remove every copy of its content (workspace files, traces, embeddings), and there is no administrator purge for spillage.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="2">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="F17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="2">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="H17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Key limits on a trusted forwarded client address, bound memory without clearing all windows, and rate-limit /api/auth/entra/login per client instead of a global cap.</t>
+          <t xml:space="preserve">Add a cascading purge with verification.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J17" t="inlineStr" s="2">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="B18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-7</t>
+          <t xml:space="preserve">SC-5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-7 Boundary Protection</t>
+          <t xml:space="preserve">SC-5 Denial-of-Service Protection</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The address check resolves DNS separately from the connection that follows, so a host that changes its DNS answer between the two can reach an internal address. The deployment Key Vault is created with public network access enabled.</t>
+          <t xml:space="preserve">Rate limits are in memory and keyed on the socket address; behind the appliance's nginx proxy every client shares one address, and the limiter clears all windows once it tracks 10,000 keys. The cap of 256 pending sign-ins can be exhausted by unauthenticated requests, blocking sign-in for up to 10 minutes.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="2">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="2">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="H18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Connect to the address that was checked (pinned lookup) for all outbound requests, and support private endpoints or firewall rules for the deployment Key Vault.</t>
+          <t xml:space="preserve">Key limits on a trusted forwarded client address, bound memory without clearing all windows, and rate-limit /api/auth/entra/login per client instead of a global cap.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr" s="2">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="B19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-12</t>
+          <t xml:space="preserve">SC-7</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-12 Cryptographic Key Establishment and Management</t>
+          <t xml:space="preserve">SC-7 Boundary Protection</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">There is no rotation or key-versioning support for the portal secret or the local master key. Encryption keys for connector credentials are derived with a single SHA-256 of the portal secret, so changing that secret makes stored values unreadable. The Key Vault uses the Standard (software-protected) tier.</t>
+          <t xml:space="preserve">The address check resolves DNS separately from the connection that follows, so a host that changes its DNS answer between the two can reach an internal address. The deployment Key Vault is created with public network access enabled.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="2">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="2">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="H19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Introduce versioned data-encryption keys with a proper KDF, a re-encryption procedure for rotation, and an option for HSM-backed keys.</t>
+          <t xml:space="preserve">Connect to the address that was checked (pinned lookup) for all outbound requests, and support private endpoints or firewall rules for the deployment Key Vault.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Before first federal pilot</t>
         </is>
       </c>
       <c r="J19" t="inlineStr" s="2">
@@ -1161,17 +1161,17 @@
       </c>
       <c r="B20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-13</t>
+          <t xml:space="preserve">SC-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-13 Cryptographic Protection</t>
+          <t xml:space="preserve">SC-12 Cryptographic Key Establishment and Management</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus does not enable OpenSSL FIPS mode or a FIPS provider, and the image is not built on a FIPS 140 validated cryptographic module. Algorithms in use are FIPS-approved, but no validated module is claimed.</t>
+          <t xml:space="preserve">There is no rotation or key-versioning support for the portal secret or the local master key. Encryption keys for connector credentials are derived with a single SHA-256 of the portal secret, so changing that secret makes stored values unreadable. The Key Vault uses the Standard (software-protected) tier.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="2">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="F20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="2">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Build a FIPS variant of the image on a FIPS 140-3 validated OpenSSL provider, enable FIPS mode at startup, fail startup if it is unavailable, and test that every code path works under it.</t>
+          <t xml:space="preserve">Introduce versioned data-encryption keys with a proper KDF, a re-encryption procedure for rotation, and an option for HSM-backed keys.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr" s="2">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="J20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">high</t>
+          <t xml:space="preserve">moderate</t>
         </is>
       </c>
       <c r="K20" t="inlineStr" s="2">
@@ -1218,17 +1218,17 @@
       </c>
       <c r="B21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-28</t>
+          <t xml:space="preserve">SC-13</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-28 Protection of Information at Rest</t>
+          <t xml:space="preserve">SC-13 Cryptographic Protection</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Agent sessions, Library documents, Resource Class records, audit logs and traces are stored in unencrypted SQLite and AgentFS files; their protection at rest depends entirely on volume encryption that Papyrus neither provides nor checks.</t>
+          <t xml:space="preserve">Signatures and MACs use P-256 and SHA-256 rather than the CNSA suite (P-384, SHA-384) that national security systems may require.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="2">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="2">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="H21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Document volume encryption as a deployment requirement and verify it on supported deployment configurations, or add database-level encryption for the main data stores.</t>
+          <t xml:space="preserve">Move Papyrus-generated signatures and MACs to CNSA algorithms while still verifying existing ones.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J21" t="inlineStr" s="2">
@@ -1275,17 +1275,17 @@
       </c>
       <c r="B22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-39</t>
+          <t xml:space="preserve">SC-28</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SC-39 Process Isolation</t>
+          <t xml:space="preserve">SC-28 Protection of Information at Rest</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The Factory sidecar, enabled by default in the image (PAPYRUS_FACTORY_SIDECAR=1), runs commands for App builds in Mastra's LocalSandbox with no kernel isolation: only its environment is restricted to an allow-list. Those commands run as the same user as the daemon, can read files that user can read, including the Papyrus data directory, and have network access.</t>
+          <t xml:space="preserve">Agent sessions, Library documents, audit records and traces are stored in unencrypted SQLite and AgentFS files; their confidentiality at rest depends on volume encryption the deploying organization provides.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="2">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="2">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="H22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Run Factory sidecar commands under the same landstrip policy as agent workspace commands (data directory denied, network denied or limited to package mirrors and source control), or disable the sidecar by default until that is in place.</t>
+          <t xml:space="preserve">Require and verify an encrypted volume for the data directory on classified deployments.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J22" t="inlineStr" s="2">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="C28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FIPS 140 validated cryptography not enabled</t>
+          <t xml:space="preserve">Vulnerability scanning and remediation SLAs not formalized</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No code, configuration or image in the repository enables OpenSSL FIPS mode or a FIPS provider. Papyrus uses FIPS-approved algorithms through Node.js crypto but does not run on a validated module.</t>
+          <t xml:space="preserve">CI performs no dependency, static or image vulnerability scanning; there are no severity-based remediation timeframes and no published vulnerability disclosure policy.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="2">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="F28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="2">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="H28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Produce a FIPS image variant on a FIPS 140-3 validated provider with FIPS mode enforced at startup (see sc-13).</t>
+          <t xml:space="preserve">Add scanning to CI (see ra-5), publish a disclosure policy, and adopt remediation SLAs such as those in the FedRAMP continuous monitoring guidance.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal ATO package</t>
+          <t xml:space="preserve">Before first federal pilot</t>
         </is>
       </c>
       <c r="J28" t="inlineStr" s="2">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="C29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vulnerability scanning and remediation SLAs not formalized</t>
+          <t xml:space="preserve">Incident response and contingency planning owned by the deploying organization</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CI performs no dependency, static or image vulnerability scanning; there are no severity-based remediation timeframes and no published vulnerability disclosure policy.</t>
+          <t xml:space="preserve">Papyrus ships no incident response plan, contingency plan, or backup tooling. Each deploying organization must cover Papyrus in its own IR and CP documentation, and Beag Labs has no published process for notifying customers of product security incidents.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="2">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="F29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="2">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="H29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add scanning to CI (see ra-5), publish a disclosure policy, and adopt remediation SLAs such as those in the FedRAMP continuous monitoring guidance.</t>
+          <t xml:space="preserve">Publish customer-facing guidance for IR and backup/restore of a Papyrus deployment and a Beag Labs product security incident notification process.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="2">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="J29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">high</t>
+          <t xml:space="preserve">moderate</t>
         </is>
       </c>
       <c r="K29" t="inlineStr" s="2">
@@ -1736,12 +1736,12 @@
       </c>
       <c r="C30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Incident response and contingency planning owned by the deploying organization</t>
+          <t xml:space="preserve">Security tests and compliance checks not enforced in CI</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus ships no incident response plan, contingency plan, or backup tooling. Each deploying organization must cover Papyrus in its own IR and CP documentation, and Beag Labs has no published process for notifying customers of product security incidents.</t>
+          <t xml:space="preserve">CI runs type checking and a subset of tests; most security tests and the compliance drift check run only locally through a pre-commit hook that can be bypassed. The generated compliance/ssp.md states that these checks also run in CI.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="2">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="2">
@@ -1761,12 +1761,12 @@
       </c>
       <c r="H30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Publish customer-facing guidance for IR and backup/restore of a Papyrus deployment and a Beag Labs product security incident notification process.</t>
+          <t xml:space="preserve">Run the full test suite and pnpm compliance:check as required CI checks, and correct the SSP text until they do (see sa-11).</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Next release</t>
         </is>
       </c>
       <c r="J30" t="inlineStr" s="2">
@@ -1793,12 +1793,12 @@
       </c>
       <c r="C31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security tests and compliance checks not enforced in CI</t>
+          <t xml:space="preserve">License signing-key custody outside assessment scope</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CI runs type checking and a subset of tests; most security tests and the compliance drift check run only locally through a pre-commit hook that can be bypassed. The generated compliance/ssp.md states that these checks also run in CI.</t>
+          <t xml:space="preserve">Licenses are signed offline with Beag Labs' Azure Key Vault keys (beag-master, beag-dev). Custody of and access to those keys is not documented here.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="2">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="H31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Run the full test suite and pnpm compliance:check as required CI checks, and correct the SSP text until they do (see sa-11).</t>
+          <t xml:space="preserve">Produce a control description for the license signing keys, including custody, access and rotation.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Next release</t>
+          <t xml:space="preserve">Before first federal pilot</t>
         </is>
       </c>
       <c r="J31" t="inlineStr" s="2">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="C32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">First-run setup is not authenticated</t>
+          <t xml:space="preserve">Agent tool lists do not limit tool use</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before identity is configured, the setup server accepts the Entra tenant and client configuration from any caller that can reach it, with no setup token, once Terms are accepted and an entitlement is present. HTTPS is required for this step only on verified Marketplace deployments in persistent mode; elsewhere setup can run over plain HTTP.</t>
+          <t xml:space="preserve">Within an active agent session any tool the deployment offers may be used; the tools listed in an agent's signed revision record intent but are not enforced. Approval prompts, budgets and channel approvals still apply.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="2">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="F32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
+          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="2">
@@ -1875,17 +1875,17 @@
       </c>
       <c r="H32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Require a one-time setup token printed to the host console or delivered through the deployment channel, and require HTTPS for setup in persistent mode on every deployment path.</t>
+          <t xml:space="preserve">Where an enclave requires per-agent least functionality, restore enforcement of the signed tool list or restrict the deployment-wide tool set.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before first federal pilot</t>
+          <t xml:space="preserve">Before first classified deployment</t>
         </is>
       </c>
       <c r="J32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">high</t>
+          <t xml:space="preserve">moderate</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
@@ -1894,121 +1894,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PAP-032</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Program</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Beag Labs control plane and license authority outside assessment scope</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Control-plane deployments trust papyrus.beaglabs.com and license.beaglabs.com to entitle and suspend them, bind their tenant and first System Owner, broker Microsoft sign-in, and issue Graph tokens. That code is not in this repository and none of its controls are documented here.</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Provider self-assessment</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Beag Labs, Inc.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Produce a separate control description for the control plane and license authority, including signing-key custody, or document the self-registration and disconnected deployment modes as the path for organizations that cannot accept the dependency.</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Before first federal pilot</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">moderate</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">PAP-033</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Program</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Security documentation does not match the implementation in places</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">compliance/ssp.md and docs/workspace-security-model.md describe the workspace sandbox as nono, while the code applies landstrip (Landlock and seccomp) through files still named workspace-nono; docs/security.md describes the current behavior.</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Provider self-assessment</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Papyrus 0.1.0+fd55e38</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Beag Labs, Inc.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Update the SSP generator text and workspace documentation to name landstrip, and rename the files.</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Next release</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">low</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K34"/>
+  <autoFilter ref="A1:K32"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Papyrus evidence pack for release 0.1.0+3e23d44
Image ghcr.io/beaglabs/papyrus/papyrus@sha256:d399de55 (built 2026-10-27): signature and SLSA
provenance verified, no critical or high findings on either platform.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/compliance/papyrus/papyrus-poam.xlsx
+++ b/public/compliance/papyrus/papyrus-poam.xlsx
@@ -155,7 +155,7 @@
       </c>
       <c r="F2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="2">
@@ -212,7 +212,7 @@
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="2">
@@ -269,7 +269,7 @@
       </c>
       <c r="F4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="2">
@@ -326,7 +326,7 @@
       </c>
       <c r="F5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="2">
@@ -383,7 +383,7 @@
       </c>
       <c r="F6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="2">
@@ -440,7 +440,7 @@
       </c>
       <c r="F7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G7" t="inlineStr" s="2">
@@ -497,7 +497,7 @@
       </c>
       <c r="F8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="2">
@@ -554,7 +554,7 @@
       </c>
       <c r="F9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G9" t="inlineStr" s="2">
@@ -611,7 +611,7 @@
       </c>
       <c r="F10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G10" t="inlineStr" s="2">
@@ -668,7 +668,7 @@
       </c>
       <c r="F11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="2">
@@ -725,7 +725,7 @@
       </c>
       <c r="F12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="2">
@@ -782,7 +782,7 @@
       </c>
       <c r="F13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="2">
@@ -839,7 +839,7 @@
       </c>
       <c r="F14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="2">
@@ -896,7 +896,7 @@
       </c>
       <c r="F15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G15" t="inlineStr" s="2">
@@ -953,7 +953,7 @@
       </c>
       <c r="F16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G16" t="inlineStr" s="2">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="F17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="2">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="2">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="2">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="F20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="2">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="2">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="2">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="F28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="2">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="F29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="2">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="2">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="F32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Papyrus 0.1.0+a3d9ded</t>
+          <t xml:space="preserve">Papyrus 0.1.0+3e23d44</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="2">

</xml_diff>